<commit_message>
Update with 103 Valid Responses
</commit_message>
<xml_diff>
--- a/305 - Research Project/05-research-data-and-analysis/03-scored-dataset/final-analysis-workbook.xlsx
+++ b/305 - Research Project/05-research-data-and-analysis/03-scored-dataset/final-analysis-workbook.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rec95d38f08544755"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eligible Data" sheetId="2" r:id="R189ec46a0767427a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eligibility Audit" sheetId="3" r:id="Rd554a3db8f6d417d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="4" r:id="R5280dee068bd4bd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R1e2ea28d08e84bfd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eligible Data" sheetId="2" r:id="R98a946bf1eeb462b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eligibility Audit" sheetId="3" r:id="Ree788a354fce4723"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="4" r:id="Rf2907be8a6274f71"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -593,7 +593,7 @@
         <x:v>Processing note</x:v>
       </x:c>
       <x:c r="B8" s="25" t="str">
-        <x:v>Two approved item imputations are retained; profile blanks remain missing</x:v>
+        <x:v>Two approved item replacements are retained; profile blanks remain missing</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -9004,42 +9004,44 @@
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="44" t="str">
-        <x:v>Manual-25</x:v>
+        <x:v>Manual-27</x:v>
       </x:c>
       <x:c r="B72" s="44" t="str">
         <x:v>manual</x:v>
       </x:c>
-      <x:c r="C72" s="44" t="str"/>
+      <x:c r="C72" s="44" t="str">
+        <x:v>45–54</x:v>
+      </x:c>
       <x:c r="D72" s="44" t="str">
-        <x:v>Above 20 years</x:v>
+        <x:v>11–20 years</x:v>
       </x:c>
       <x:c r="E72" s="44" t="str">
         <x:v>Clerical</x:v>
       </x:c>
       <x:c r="F72" s="45" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G72" s="45" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H72" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I72" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="J72" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="K72" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L72" s="46" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="M72" s="46" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="M72" s="46" t="n">
-        <x:v>3.333</x:v>
-      </x:c>
       <x:c r="N72" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -9053,7 +9055,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="R72" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="S72" s="46" t="n">
         <x:v>4</x:v>
@@ -9068,7 +9070,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="W72" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="X72" s="46" t="n">
         <x:v>4</x:v>
@@ -9077,7 +9079,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="Z72" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AA72" s="46" t="n">
         <x:v>4</x:v>
@@ -9092,7 +9094,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="AE72" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AF72" s="46" t="n">
         <x:v>4</x:v>
@@ -9102,36 +9104,36 @@
       </x:c>
       <x:c r="AH72" s="46" t="n">
         <x:f>AVERAGE(H72:N72)</x:f>
-        <x:v>3.333285714285714</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AI72" s="46" t="n">
         <x:f>AVERAGE(O72:T72)</x:f>
-        <x:v>4</x:v>
+        <x:v>3.6666666666666665</x:v>
       </x:c>
       <x:c r="AJ72" s="46" t="n">
         <x:f>AVERAGE(U72:Z72)</x:f>
-        <x:v>3.8333333333333335</x:v>
+        <x:v>4.333333333333333</x:v>
       </x:c>
       <x:c r="AK72" s="46" t="n">
         <x:f>AVERAGE(AA72:AG72)</x:f>
-        <x:v>4</x:v>
+        <x:v>4.142857142857143</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="44" t="str">
-        <x:v>Manual-27</x:v>
+        <x:v>Manual-28</x:v>
       </x:c>
       <x:c r="B73" s="44" t="str">
         <x:v>manual</x:v>
       </x:c>
       <x:c r="C73" s="44" t="str">
-        <x:v>45–54</x:v>
+        <x:v>35–44</x:v>
       </x:c>
       <x:c r="D73" s="44" t="str">
         <x:v>11–20 years</x:v>
       </x:c>
       <x:c r="E73" s="44" t="str">
-        <x:v>Clerical</x:v>
+        <x:v>Officer</x:v>
       </x:c>
       <x:c r="F73" s="45" t="n">
         <x:v>0</x:v>
@@ -9149,28 +9151,28 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="K73" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L73" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="M73" s="46" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="N73" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="O73" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="P73" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Q73" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="R73" s="46" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="S73" s="46" t="n">
         <x:v>4</x:v>
@@ -9182,7 +9184,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="V73" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="W73" s="46" t="n">
         <x:v>5</x:v>
@@ -9191,7 +9193,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="Y73" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Z73" s="46" t="n">
         <x:v>5</x:v>
@@ -9200,13 +9202,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="AB73" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AC73" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AD73" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AE73" s="46" t="n">
         <x:v>5</x:v>
@@ -9219,24 +9221,24 @@
       </x:c>
       <x:c r="AH73" s="46" t="n">
         <x:f>AVERAGE(H73:N73)</x:f>
-        <x:v>4</x:v>
+        <x:v>4.428571428571429</x:v>
       </x:c>
       <x:c r="AI73" s="46" t="n">
         <x:f>AVERAGE(O73:T73)</x:f>
-        <x:v>3.6666666666666665</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="AJ73" s="46" t="n">
         <x:f>AVERAGE(U73:Z73)</x:f>
-        <x:v>4.333333333333333</x:v>
+        <x:v>4.666666666666667</x:v>
       </x:c>
       <x:c r="AK73" s="46" t="n">
         <x:f>AVERAGE(AA73:AG73)</x:f>
-        <x:v>4.142857142857143</x:v>
+        <x:v>4.571428571428571</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="44" t="str">
-        <x:v>Manual-28</x:v>
+        <x:v>Manual-29</x:v>
       </x:c>
       <x:c r="B74" s="44" t="str">
         <x:v>manual</x:v>
@@ -9248,7 +9250,7 @@
         <x:v>11–20 years</x:v>
       </x:c>
       <x:c r="E74" s="44" t="str">
-        <x:v>Officer</x:v>
+        <x:v>Clerical</x:v>
       </x:c>
       <x:c r="F74" s="45" t="n">
         <x:v>0</x:v>
@@ -9257,7 +9259,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H74" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="I74" s="46" t="n">
         <x:v>4</x:v>
@@ -9266,13 +9268,13 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="K74" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L74" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="M74" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="N74" s="46" t="n">
         <x:v>5</x:v>
@@ -9284,22 +9286,22 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="Q74" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="R74" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="S74" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T74" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="U74" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="V74" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="W74" s="46" t="n">
         <x:v>5</x:v>
@@ -9314,13 +9316,13 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="AA74" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AB74" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="AC74" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AD74" s="46" t="n">
         <x:v>5</x:v>
@@ -9332,15 +9334,15 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="AG74" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AH74" s="46" t="n">
         <x:f>AVERAGE(H74:N74)</x:f>
-        <x:v>4.428571428571429</x:v>
+        <x:v>4.714285714285714</x:v>
       </x:c>
       <x:c r="AI74" s="46" t="n">
         <x:f>AVERAGE(O74:T74)</x:f>
-        <x:v>4.5</x:v>
+        <x:v>4.833333333333333</x:v>
       </x:c>
       <x:c r="AJ74" s="46" t="n">
         <x:f>AVERAGE(U74:Z74)</x:f>
@@ -9348,12 +9350,12 @@
       </x:c>
       <x:c r="AK74" s="46" t="n">
         <x:f>AVERAGE(AA74:AG74)</x:f>
-        <x:v>4.571428571428571</x:v>
+        <x:v>4.714285714285714</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="44" t="str">
-        <x:v>Manual-29</x:v>
+        <x:v>Manual-30</x:v>
       </x:c>
       <x:c r="B75" s="44" t="str">
         <x:v>manual</x:v>
@@ -9362,10 +9364,10 @@
         <x:v>35–44</x:v>
       </x:c>
       <x:c r="D75" s="44" t="str">
-        <x:v>11–20 years</x:v>
+        <x:v>5–10 years</x:v>
       </x:c>
       <x:c r="E75" s="44" t="str">
-        <x:v>Clerical</x:v>
+        <x:v>Officer</x:v>
       </x:c>
       <x:c r="F75" s="45" t="n">
         <x:v>0</x:v>
@@ -9374,13 +9376,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H75" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I75" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="J75" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="K75" s="46" t="n">
         <x:v>5</x:v>
@@ -9395,49 +9397,49 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="O75" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="P75" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="Q75" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="R75" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="S75" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="T75" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="U75" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="V75" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="W75" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="X75" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="Y75" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Z75" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AA75" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AB75" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="AC75" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AD75" s="46" t="n">
         <x:v>5</x:v>
@@ -9446,43 +9448,43 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="AF75" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AG75" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="AH75" s="46" t="n">
         <x:f>AVERAGE(H75:N75)</x:f>
-        <x:v>4.714285714285714</x:v>
+        <x:v>4.428571428571429</x:v>
       </x:c>
       <x:c r="AI75" s="46" t="n">
         <x:f>AVERAGE(O75:T75)</x:f>
-        <x:v>4.833333333333333</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="AJ75" s="46" t="n">
         <x:f>AVERAGE(U75:Z75)</x:f>
-        <x:v>4.666666666666667</x:v>
+        <x:v>4.333333333333333</x:v>
       </x:c>
       <x:c r="AK75" s="46" t="n">
         <x:f>AVERAGE(AA75:AG75)</x:f>
-        <x:v>4.714285714285714</x:v>
+        <x:v>4.857142857142857</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="44" t="str">
-        <x:v>Manual-30</x:v>
+        <x:v>Manual-31</x:v>
       </x:c>
       <x:c r="B76" s="44" t="str">
         <x:v>manual</x:v>
       </x:c>
       <x:c r="C76" s="44" t="str">
-        <x:v>35–44</x:v>
+        <x:v>25–34</x:v>
       </x:c>
       <x:c r="D76" s="44" t="str">
-        <x:v>5–10 years</x:v>
+        <x:v>11–20 years</x:v>
       </x:c>
       <x:c r="E76" s="44" t="str">
-        <x:v>Officer</x:v>
+        <x:v>Clerical</x:v>
       </x:c>
       <x:c r="F76" s="45" t="n">
         <x:v>0</x:v>
@@ -9491,7 +9493,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H76" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="I76" s="46" t="n">
         <x:v>4</x:v>
@@ -9503,7 +9505,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="L76" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="M76" s="46" t="n">
         <x:v>5</x:v>
@@ -9515,13 +9517,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="P76" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Q76" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="R76" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="S76" s="46" t="n">
         <x:v>4</x:v>
@@ -9536,19 +9538,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="W76" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="X76" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Y76" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Z76" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AA76" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AB76" s="46" t="n">
         <x:v>5</x:v>
@@ -9570,36 +9572,36 @@
       </x:c>
       <x:c r="AH76" s="46" t="n">
         <x:f>AVERAGE(H76:N76)</x:f>
-        <x:v>4.428571428571429</x:v>
+        <x:v>4.714285714285714</x:v>
       </x:c>
       <x:c r="AI76" s="46" t="n">
         <x:f>AVERAGE(O76:T76)</x:f>
-        <x:v>4.5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AJ76" s="46" t="n">
         <x:f>AVERAGE(U76:Z76)</x:f>
-        <x:v>4.333333333333333</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AK76" s="46" t="n">
         <x:f>AVERAGE(AA76:AG76)</x:f>
-        <x:v>4.857142857142857</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="44" t="str">
-        <x:v>Manual-31</x:v>
+        <x:v>Manual-33</x:v>
       </x:c>
       <x:c r="B77" s="44" t="str">
         <x:v>manual</x:v>
       </x:c>
       <x:c r="C77" s="44" t="str">
-        <x:v>25–34</x:v>
+        <x:v>35–44</x:v>
       </x:c>
       <x:c r="D77" s="44" t="str">
         <x:v>11–20 years</x:v>
       </x:c>
       <x:c r="E77" s="44" t="str">
-        <x:v>Clerical</x:v>
+        <x:v>Managerial</x:v>
       </x:c>
       <x:c r="F77" s="45" t="n">
         <x:v>0</x:v>
@@ -9611,10 +9613,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="I77" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J77" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="K77" s="46" t="n">
         <x:v>5</x:v>
@@ -9632,7 +9634,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="P77" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Q77" s="46" t="n">
         <x:v>4</x:v>
@@ -9647,64 +9649,64 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="U77" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="V77" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="W77" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="X77" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Y77" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Z77" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AA77" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AB77" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AC77" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AD77" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AE77" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AF77" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AG77" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AH77" s="46" t="n">
         <x:f>AVERAGE(H77:N77)</x:f>
-        <x:v>4.714285714285714</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AI77" s="46" t="n">
         <x:f>AVERAGE(O77:T77)</x:f>
-        <x:v>4</x:v>
+        <x:v>4.166666666666667</x:v>
       </x:c>
       <x:c r="AJ77" s="46" t="n">
         <x:f>AVERAGE(U77:Z77)</x:f>
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AK77" s="46" t="n">
         <x:f>AVERAGE(AA77:AG77)</x:f>
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="44" t="str">
-        <x:v>Manual-33</x:v>
+        <x:v>Manual-35</x:v>
       </x:c>
       <x:c r="B78" s="44" t="str">
         <x:v>manual</x:v>
@@ -9716,7 +9718,7 @@
         <x:v>11–20 years</x:v>
       </x:c>
       <x:c r="E78" s="44" t="str">
-        <x:v>Managerial</x:v>
+        <x:v>Officer</x:v>
       </x:c>
       <x:c r="F78" s="45" t="n">
         <x:v>0</x:v>
@@ -9725,31 +9727,31 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H78" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I78" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J78" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="K78" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L78" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="M78" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="N78" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="O78" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="P78" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Q78" s="46" t="n">
         <x:v>4</x:v>
@@ -9758,10 +9760,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="S78" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="T78" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="U78" s="46" t="n">
         <x:v>4</x:v>
@@ -9776,7 +9778,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="Y78" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="Z78" s="46" t="n">
         <x:v>4</x:v>
@@ -9788,7 +9790,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="AC78" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AD78" s="46" t="n">
         <x:v>4</x:v>
@@ -9804,24 +9806,24 @@
       </x:c>
       <x:c r="AH78" s="46" t="n">
         <x:f>AVERAGE(H78:N78)</x:f>
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AI78" s="46" t="n">
         <x:f>AVERAGE(O78:T78)</x:f>
-        <x:v>4.166666666666667</x:v>
+        <x:v>3.6666666666666665</x:v>
       </x:c>
       <x:c r="AJ78" s="46" t="n">
         <x:f>AVERAGE(U78:Z78)</x:f>
-        <x:v>4</x:v>
+        <x:v>3.8333333333333335</x:v>
       </x:c>
       <x:c r="AK78" s="46" t="n">
         <x:f>AVERAGE(AA78:AG78)</x:f>
-        <x:v>4</x:v>
+        <x:v>4.142857142857143</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="44" t="str">
-        <x:v>Manual-35</x:v>
+        <x:v>Manual-36</x:v>
       </x:c>
       <x:c r="B79" s="44" t="str">
         <x:v>manual</x:v>
@@ -9830,7 +9832,7 @@
         <x:v>35–44</x:v>
       </x:c>
       <x:c r="D79" s="44" t="str">
-        <x:v>11–20 years</x:v>
+        <x:v>5–10 years</x:v>
       </x:c>
       <x:c r="E79" s="44" t="str">
         <x:v>Officer</x:v>
@@ -9842,115 +9844,115 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H79" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="I79" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J79" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="K79" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L79" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="M79" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="N79" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="O79" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="P79" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="Q79" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="R79" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="S79" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T79" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="U79" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="V79" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="W79" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="X79" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Y79" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Z79" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AA79" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AB79" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AC79" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="AD79" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AE79" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AF79" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AG79" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AH79" s="46" t="n">
         <x:f>AVERAGE(H79:N79)</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AI79" s="46" t="n">
         <x:f>AVERAGE(O79:T79)</x:f>
-        <x:v>3.6666666666666665</x:v>
+        <x:v>4.833333333333333</x:v>
       </x:c>
       <x:c r="AJ79" s="46" t="n">
         <x:f>AVERAGE(U79:Z79)</x:f>
-        <x:v>3.8333333333333335</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AK79" s="46" t="n">
         <x:f>AVERAGE(AA79:AG79)</x:f>
-        <x:v>4.142857142857143</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="44" t="str">
-        <x:v>Manual-36</x:v>
+        <x:v>Manual-38</x:v>
       </x:c>
       <x:c r="B80" s="44" t="str">
         <x:v>manual</x:v>
       </x:c>
       <x:c r="C80" s="44" t="str">
-        <x:v>35–44</x:v>
+        <x:v>55 and above</x:v>
       </x:c>
       <x:c r="D80" s="44" t="str">
-        <x:v>5–10 years</x:v>
+        <x:v>11–20 years</x:v>
       </x:c>
       <x:c r="E80" s="44" t="str">
-        <x:v>Officer</x:v>
+        <x:v>Managerial</x:v>
       </x:c>
       <x:c r="F80" s="45" t="n">
         <x:v>0</x:v>
@@ -9968,7 +9970,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="K80" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L80" s="46" t="n">
         <x:v>5</x:v>
@@ -9983,7 +9985,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="P80" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Q80" s="46" t="n">
         <x:v>5</x:v>
@@ -10001,13 +10003,13 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="V80" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="W80" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="X80" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Y80" s="46" t="n">
         <x:v>5</x:v>
@@ -10025,45 +10027,49 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="AD80" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AE80" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AF80" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AG80" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="AH80" s="46" t="n">
         <x:f>AVERAGE(H80:N80)</x:f>
-        <x:v>5</x:v>
+        <x:v>4.857142857142857</x:v>
       </x:c>
       <x:c r="AI80" s="46" t="n">
         <x:f>AVERAGE(O80:T80)</x:f>
-        <x:v>4.833333333333333</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AJ80" s="46" t="n">
         <x:f>AVERAGE(U80:Z80)</x:f>
-        <x:v>5</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="AK80" s="46" t="n">
         <x:f>AVERAGE(AA80:AG80)</x:f>
-        <x:v>5</x:v>
+        <x:v>4.571428571428571</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="44" t="str">
-        <x:v>Manual-37</x:v>
+        <x:v>Manual-39</x:v>
       </x:c>
       <x:c r="B81" s="44" t="str">
         <x:v>manual</x:v>
       </x:c>
-      <x:c r="C81" s="44" t="str"/>
-      <x:c r="D81" s="44" t="str"/>
+      <x:c r="C81" s="44" t="str">
+        <x:v>35–44</x:v>
+      </x:c>
+      <x:c r="D81" s="44" t="str">
+        <x:v>11–20 years</x:v>
+      </x:c>
       <x:c r="E81" s="44" t="str">
-        <x:v>Clerical</x:v>
+        <x:v>Officer</x:v>
       </x:c>
       <x:c r="F81" s="45" t="n">
         <x:v>0</x:v>
@@ -10075,22 +10081,22 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="I81" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J81" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="K81" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L81" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="M81" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="N81" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="O81" s="46" t="n">
         <x:v>5</x:v>
@@ -10099,16 +10105,16 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="Q81" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="R81" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="S81" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="T81" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="U81" s="46" t="n">
         <x:v>5</x:v>
@@ -10132,7 +10138,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="AB81" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AC81" s="46" t="n">
         <x:v>5</x:v>
@@ -10144,18 +10150,18 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="AF81" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AG81" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AH81" s="46" t="n">
         <x:f>AVERAGE(H81:N81)</x:f>
-        <x:v>4.714285714285714</x:v>
+        <x:v>4.285714285714286</x:v>
       </x:c>
       <x:c r="AI81" s="46" t="n">
         <x:f>AVERAGE(O81:T81)</x:f>
-        <x:v>4.666666666666667</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="AJ81" s="46" t="n">
         <x:f>AVERAGE(U81:Z81)</x:f>
@@ -10163,24 +10169,24 @@
       </x:c>
       <x:c r="AK81" s="46" t="n">
         <x:f>AVERAGE(AA81:AG81)</x:f>
-        <x:v>4.571428571428571</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="44" t="str">
-        <x:v>Manual-38</x:v>
+        <x:v>Manual-41</x:v>
       </x:c>
       <x:c r="B82" s="44" t="str">
         <x:v>manual</x:v>
       </x:c>
       <x:c r="C82" s="44" t="str">
-        <x:v>55 and above</x:v>
+        <x:v>35–44</x:v>
       </x:c>
       <x:c r="D82" s="44" t="str">
-        <x:v>11–20 years</x:v>
+        <x:v>Below 5 years</x:v>
       </x:c>
       <x:c r="E82" s="44" t="str">
-        <x:v>Managerial</x:v>
+        <x:v>Officer</x:v>
       </x:c>
       <x:c r="F82" s="45" t="n">
         <x:v>0</x:v>
@@ -10195,10 +10201,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="J82" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="K82" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L82" s="46" t="n">
         <x:v>5</x:v>
@@ -10210,10 +10216,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="O82" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="P82" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Q82" s="46" t="n">
         <x:v>5</x:v>
@@ -10228,7 +10234,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="U82" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="V82" s="46" t="n">
         <x:v>4</x:v>
@@ -10237,7 +10243,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="X82" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Y82" s="46" t="n">
         <x:v>5</x:v>
@@ -10255,13 +10261,13 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="AD82" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AE82" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AF82" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AG82" s="46" t="n">
         <x:v>5</x:v>
@@ -10272,7 +10278,7 @@
       </x:c>
       <x:c r="AI82" s="46" t="n">
         <x:f>AVERAGE(O82:T82)</x:f>
-        <x:v>5</x:v>
+        <x:v>4.666666666666667</x:v>
       </x:c>
       <x:c r="AJ82" s="46" t="n">
         <x:f>AVERAGE(U82:Z82)</x:f>
@@ -10280,24 +10286,24 @@
       </x:c>
       <x:c r="AK82" s="46" t="n">
         <x:f>AVERAGE(AA82:AG82)</x:f>
-        <x:v>4.571428571428571</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="44" t="str">
-        <x:v>Manual-39</x:v>
+        <x:v>Manual-42</x:v>
       </x:c>
       <x:c r="B83" s="44" t="str">
         <x:v>manual</x:v>
       </x:c>
       <x:c r="C83" s="44" t="str">
-        <x:v>35–44</x:v>
+        <x:v>25–34</x:v>
       </x:c>
       <x:c r="D83" s="44" t="str">
-        <x:v>11–20 years</x:v>
+        <x:v>5–10 years</x:v>
       </x:c>
       <x:c r="E83" s="44" t="str">
-        <x:v>Officer</x:v>
+        <x:v>Clerical</x:v>
       </x:c>
       <x:c r="F83" s="45" t="n">
         <x:v>0</x:v>
@@ -10309,22 +10315,22 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="I83" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J83" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="K83" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L83" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="M83" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="N83" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="O83" s="46" t="n">
         <x:v>5</x:v>
@@ -10336,13 +10342,13 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="R83" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="S83" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T83" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="U83" s="46" t="n">
         <x:v>5</x:v>
@@ -10354,16 +10360,16 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="X83" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Y83" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Z83" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="AA83" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AB83" s="46" t="n">
         <x:v>5</x:v>
@@ -10375,7 +10381,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="AE83" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AF83" s="46" t="n">
         <x:v>5</x:v>
@@ -10385,57 +10391,57 @@
       </x:c>
       <x:c r="AH83" s="46" t="n">
         <x:f>AVERAGE(H83:N83)</x:f>
-        <x:v>4.285714285714286</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AI83" s="46" t="n">
         <x:f>AVERAGE(O83:T83)</x:f>
-        <x:v>4.5</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AJ83" s="46" t="n">
         <x:f>AVERAGE(U83:Z83)</x:f>
-        <x:v>5</x:v>
+        <x:v>4.666666666666667</x:v>
       </x:c>
       <x:c r="AK83" s="46" t="n">
         <x:f>AVERAGE(AA83:AG83)</x:f>
-        <x:v>5</x:v>
+        <x:v>4.714285714285714</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="44" t="str">
-        <x:v>Manual-41</x:v>
+        <x:v>Manual-46</x:v>
       </x:c>
       <x:c r="B84" s="44" t="str">
         <x:v>manual</x:v>
       </x:c>
       <x:c r="C84" s="44" t="str">
-        <x:v>35–44</x:v>
+        <x:v>25–34</x:v>
       </x:c>
       <x:c r="D84" s="44" t="str">
-        <x:v>Below 5 years</x:v>
+        <x:v>5–10 years</x:v>
       </x:c>
       <x:c r="E84" s="44" t="str">
         <x:v>Officer</x:v>
       </x:c>
       <x:c r="F84" s="45" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G84" s="45" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H84" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I84" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J84" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="K84" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L84" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="M84" s="46" t="n">
         <x:v>5</x:v>
@@ -10450,76 +10456,76 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="Q84" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="R84" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="S84" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="T84" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="U84" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="V84" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="W84" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="X84" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="Y84" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Z84" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AA84" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AB84" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AC84" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AD84" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AE84" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AF84" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AG84" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AH84" s="46" t="n">
         <x:f>AVERAGE(H84:N84)</x:f>
-        <x:v>4.857142857142857</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AI84" s="46" t="n">
         <x:f>AVERAGE(O84:T84)</x:f>
-        <x:v>4.666666666666667</x:v>
+        <x:v>3.8333333333333335</x:v>
       </x:c>
       <x:c r="AJ84" s="46" t="n">
         <x:f>AVERAGE(U84:Z84)</x:f>
-        <x:v>4.5</x:v>
+        <x:v>3.1666666666666665</x:v>
       </x:c>
       <x:c r="AK84" s="46" t="n">
         <x:f>AVERAGE(AA84:AG84)</x:f>
-        <x:v>5</x:v>
+        <x:v>3.7142857142857144</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="44" t="str">
-        <x:v>Manual-42</x:v>
+        <x:v>Manual-47</x:v>
       </x:c>
       <x:c r="B85" s="44" t="str">
         <x:v>manual</x:v>
@@ -10531,7 +10537,7 @@
         <x:v>5–10 years</x:v>
       </x:c>
       <x:c r="E85" s="44" t="str">
-        <x:v>Clerical</x:v>
+        <x:v>Officer</x:v>
       </x:c>
       <x:c r="F85" s="45" t="n">
         <x:v>0</x:v>
@@ -10540,13 +10546,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H85" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I85" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J85" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="K85" s="46" t="n">
         <x:v>5</x:v>
@@ -10555,37 +10561,37 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="M85" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="N85" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="O85" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="P85" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Q85" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="R85" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="S85" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="T85" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="U85" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="V85" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="W85" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="X85" s="46" t="n">
         <x:v>4</x:v>
@@ -10594,55 +10600,55 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="Z85" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AA85" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AB85" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AC85" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AD85" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AE85" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="AF85" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AG85" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AH85" s="46" t="n">
         <x:f>AVERAGE(H85:N85)</x:f>
-        <x:v>5</x:v>
+        <x:v>4.285714285714286</x:v>
       </x:c>
       <x:c r="AI85" s="46" t="n">
         <x:f>AVERAGE(O85:T85)</x:f>
-        <x:v>5</x:v>
+        <x:v>4.166666666666667</x:v>
       </x:c>
       <x:c r="AJ85" s="46" t="n">
         <x:f>AVERAGE(U85:Z85)</x:f>
-        <x:v>4.666666666666667</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AK85" s="46" t="n">
         <x:f>AVERAGE(AA85:AG85)</x:f>
-        <x:v>4.714285714285714</x:v>
+        <x:v>4.142857142857143</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="44" t="str">
-        <x:v>Manual-46</x:v>
+        <x:v>Manual-48</x:v>
       </x:c>
       <x:c r="B86" s="44" t="str">
         <x:v>manual</x:v>
       </x:c>
       <x:c r="C86" s="44" t="str">
-        <x:v>25–34</x:v>
+        <x:v>35–44</x:v>
       </x:c>
       <x:c r="D86" s="44" t="str">
         <x:v>5–10 years</x:v>
@@ -10651,7 +10657,7 @@
         <x:v>Officer</x:v>
       </x:c>
       <x:c r="F86" s="45" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G86" s="45" t="n">
         <x:v>0</x:v>
@@ -10663,19 +10669,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J86" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K86" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="L86" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="M86" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="N86" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="O86" s="46" t="n">
         <x:v>4</x:v>
@@ -10690,40 +10696,40 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="S86" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="T86" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="U86" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="V86" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="W86" s="46" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="X86" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Y86" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="Z86" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AA86" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="AB86" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AC86" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="AD86" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AE86" s="46" t="n">
         <x:v>4</x:v>
@@ -10736,36 +10742,36 @@
       </x:c>
       <x:c r="AH86" s="46" t="n">
         <x:f>AVERAGE(H86:N86)</x:f>
-        <x:v>4</x:v>
+        <x:v>3.7142857142857144</x:v>
       </x:c>
       <x:c r="AI86" s="46" t="n">
         <x:f>AVERAGE(O86:T86)</x:f>
-        <x:v>3.8333333333333335</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AJ86" s="46" t="n">
         <x:f>AVERAGE(U86:Z86)</x:f>
-        <x:v>3.1666666666666665</x:v>
+        <x:v>3.6666666666666665</x:v>
       </x:c>
       <x:c r="AK86" s="46" t="n">
         <x:f>AVERAGE(AA86:AG86)</x:f>
-        <x:v>3.7142857142857144</x:v>
+        <x:v>3.4285714285714284</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="44" t="str">
-        <x:v>Manual-47</x:v>
+        <x:v>Manual-50</x:v>
       </x:c>
       <x:c r="B87" s="44" t="str">
         <x:v>manual</x:v>
       </x:c>
       <x:c r="C87" s="44" t="str">
-        <x:v>25–34</x:v>
+        <x:v>55 and above</x:v>
       </x:c>
       <x:c r="D87" s="44" t="str">
-        <x:v>5–10 years</x:v>
+        <x:v>11–20 years</x:v>
       </x:c>
       <x:c r="E87" s="44" t="str">
-        <x:v>Officer</x:v>
+        <x:v>Managerial</x:v>
       </x:c>
       <x:c r="F87" s="45" t="n">
         <x:v>0</x:v>
@@ -10786,16 +10792,16 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="L87" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="M87" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="N87" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="O87" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="P87" s="46" t="n">
         <x:v>4</x:v>
@@ -10810,13 +10816,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="T87" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="U87" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="V87" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="W87" s="46" t="n">
         <x:v>4</x:v>
@@ -10831,13 +10837,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="AA87" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AB87" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AC87" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AD87" s="46" t="n">
         <x:v>4</x:v>
@@ -10853,7 +10859,7 @@
       </x:c>
       <x:c r="AH87" s="46" t="n">
         <x:f>AVERAGE(H87:N87)</x:f>
-        <x:v>4.285714285714286</x:v>
+        <x:v>4.428571428571429</x:v>
       </x:c>
       <x:c r="AI87" s="46" t="n">
         <x:f>AVERAGE(O87:T87)</x:f>
@@ -10861,16 +10867,16 @@
       </x:c>
       <x:c r="AJ87" s="46" t="n">
         <x:f>AVERAGE(U87:Z87)</x:f>
-        <x:v>4</x:v>
+        <x:v>3.6666666666666665</x:v>
       </x:c>
       <x:c r="AK87" s="46" t="n">
         <x:f>AVERAGE(AA87:AG87)</x:f>
-        <x:v>4.142857142857143</x:v>
+        <x:v>3.7142857142857144</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="44" t="str">
-        <x:v>Manual-48</x:v>
+        <x:v>Manual-51</x:v>
       </x:c>
       <x:c r="B88" s="44" t="str">
         <x:v>manual</x:v>
@@ -10879,7 +10885,7 @@
         <x:v>35–44</x:v>
       </x:c>
       <x:c r="D88" s="44" t="str">
-        <x:v>5–10 years</x:v>
+        <x:v>11–20 years</x:v>
       </x:c>
       <x:c r="E88" s="44" t="str">
         <x:v>Officer</x:v>
@@ -10891,112 +10897,112 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H88" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="I88" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J88" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="K88" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L88" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="M88" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="N88" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="O88" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="P88" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Q88" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="R88" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="S88" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T88" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="U88" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="V88" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="W88" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="X88" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Y88" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Z88" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AA88" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AB88" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AC88" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AD88" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AE88" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AF88" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AG88" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AH88" s="46" t="n">
         <x:f>AVERAGE(H88:N88)</x:f>
-        <x:v>3.7142857142857144</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AI88" s="46" t="n">
         <x:f>AVERAGE(O88:T88)</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AJ88" s="46" t="n">
         <x:f>AVERAGE(U88:Z88)</x:f>
-        <x:v>3.6666666666666665</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AK88" s="46" t="n">
         <x:f>AVERAGE(AA88:AG88)</x:f>
-        <x:v>3.4285714285714284</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="44" t="str">
-        <x:v>Manual-50</x:v>
+        <x:v>Manual-52</x:v>
       </x:c>
       <x:c r="B89" s="44" t="str">
         <x:v>manual</x:v>
       </x:c>
       <x:c r="C89" s="44" t="str">
-        <x:v>55 and above</x:v>
+        <x:v>45–54</x:v>
       </x:c>
       <x:c r="D89" s="44" t="str">
-        <x:v>11–20 years</x:v>
+        <x:v>Above 20 years</x:v>
       </x:c>
       <x:c r="E89" s="44" t="str">
         <x:v>Managerial</x:v>
@@ -11008,19 +11014,19 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H89" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="I89" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J89" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="K89" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="L89" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="M89" s="46" t="n">
         <x:v>5</x:v>
@@ -11029,82 +11035,82 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="O89" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="P89" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Q89" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="R89" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="S89" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T89" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="U89" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="V89" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="W89" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="X89" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Y89" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Z89" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AA89" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AB89" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AC89" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AD89" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AE89" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AF89" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AG89" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AH89" s="46" t="n">
         <x:f>AVERAGE(H89:N89)</x:f>
-        <x:v>4.428571428571429</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AI89" s="46" t="n">
         <x:f>AVERAGE(O89:T89)</x:f>
-        <x:v>4.166666666666667</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AJ89" s="46" t="n">
         <x:f>AVERAGE(U89:Z89)</x:f>
-        <x:v>3.6666666666666665</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AK89" s="46" t="n">
         <x:f>AVERAGE(AA89:AG89)</x:f>
-        <x:v>3.7142857142857144</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="44" t="str">
-        <x:v>Manual-51</x:v>
+        <x:v>Manual-53</x:v>
       </x:c>
       <x:c r="B90" s="44" t="str">
         <x:v>manual</x:v>
@@ -11221,19 +11227,19 @@
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="44" t="str">
-        <x:v>Manual-52</x:v>
+        <x:v>Manual-54</x:v>
       </x:c>
       <x:c r="B91" s="44" t="str">
         <x:v>manual</x:v>
       </x:c>
       <x:c r="C91" s="44" t="str">
-        <x:v>45–54</x:v>
+        <x:v>25–34</x:v>
       </x:c>
       <x:c r="D91" s="44" t="str">
-        <x:v>Above 20 years</x:v>
+        <x:v>5–10 years</x:v>
       </x:c>
       <x:c r="E91" s="44" t="str">
-        <x:v>Managerial</x:v>
+        <x:v>Officer</x:v>
       </x:c>
       <x:c r="F91" s="45" t="n">
         <x:v>0</x:v>
@@ -11248,7 +11254,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="J91" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="K91" s="46" t="n">
         <x:v>5</x:v>
@@ -11260,13 +11266,13 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="N91" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="O91" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="P91" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Q91" s="46" t="n">
         <x:v>5</x:v>
@@ -11275,40 +11281,40 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="S91" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="T91" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="U91" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="V91" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="W91" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="X91" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Y91" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Z91" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AA91" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AB91" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AC91" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AD91" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AE91" s="46" t="n">
         <x:v>5</x:v>
@@ -11317,37 +11323,37 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="AG91" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AH91" s="46" t="n">
         <x:f>AVERAGE(H91:N91)</x:f>
-        <x:v>5</x:v>
+        <x:v>4.714285714285714</x:v>
       </x:c>
       <x:c r="AI91" s="46" t="n">
         <x:f>AVERAGE(O91:T91)</x:f>
-        <x:v>5</x:v>
+        <x:v>4.333333333333333</x:v>
       </x:c>
       <x:c r="AJ91" s="46" t="n">
         <x:f>AVERAGE(U91:Z91)</x:f>
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AK91" s="46" t="n">
         <x:f>AVERAGE(AA91:AG91)</x:f>
-        <x:v>5</x:v>
+        <x:v>4.285714285714286</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="44" t="str">
-        <x:v>Manual-53</x:v>
+        <x:v>Manual-55</x:v>
       </x:c>
       <x:c r="B92" s="44" t="str">
         <x:v>manual</x:v>
       </x:c>
       <x:c r="C92" s="44" t="str">
-        <x:v>35–44</x:v>
+        <x:v>45–54</x:v>
       </x:c>
       <x:c r="D92" s="44" t="str">
-        <x:v>11–20 years</x:v>
+        <x:v>Above 20 years</x:v>
       </x:c>
       <x:c r="E92" s="44" t="str">
         <x:v>Officer</x:v>
@@ -11362,67 +11368,67 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="I92" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J92" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="K92" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L92" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="M92" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="N92" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="O92" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="P92" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="Q92" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="R92" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="S92" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="T92" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="U92" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="V92" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="W92" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="X92" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="Y92" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Z92" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AA92" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AB92" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="AC92" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AD92" s="46" t="n">
         <x:v>5</x:v>
@@ -11438,24 +11444,24 @@
       </x:c>
       <x:c r="AH92" s="46" t="n">
         <x:f>AVERAGE(H92:N92)</x:f>
-        <x:v>5</x:v>
+        <x:v>4.285714285714286</x:v>
       </x:c>
       <x:c r="AI92" s="46" t="n">
         <x:f>AVERAGE(O92:T92)</x:f>
-        <x:v>5</x:v>
+        <x:v>4.333333333333333</x:v>
       </x:c>
       <x:c r="AJ92" s="46" t="n">
         <x:f>AVERAGE(U92:Z92)</x:f>
-        <x:v>5</x:v>
+        <x:v>4.333333333333333</x:v>
       </x:c>
       <x:c r="AK92" s="46" t="n">
         <x:f>AVERAGE(AA92:AG92)</x:f>
-        <x:v>5</x:v>
+        <x:v>4.714285714285714</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="44" t="str">
-        <x:v>Manual-54</x:v>
+        <x:v>Manual-56</x:v>
       </x:c>
       <x:c r="B93" s="44" t="str">
         <x:v>manual</x:v>
@@ -11464,7 +11470,7 @@
         <x:v>25–34</x:v>
       </x:c>
       <x:c r="D93" s="44" t="str">
-        <x:v>5–10 years</x:v>
+        <x:v>Below 5 years</x:v>
       </x:c>
       <x:c r="E93" s="44" t="str">
         <x:v>Officer</x:v>
@@ -11476,25 +11482,25 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H93" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I93" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J93" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K93" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L93" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="M93" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N93" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="O93" s="46" t="n">
         <x:v>4</x:v>
@@ -11503,16 +11509,16 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="Q93" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="R93" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="S93" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="T93" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="U93" s="46" t="n">
         <x:v>4</x:v>
@@ -11536,30 +11542,30 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="AB93" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AC93" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AD93" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="AE93" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AF93" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AG93" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AH93" s="46" t="n">
         <x:f>AVERAGE(H93:N93)</x:f>
-        <x:v>4.714285714285714</x:v>
+        <x:v>2.857142857142857</x:v>
       </x:c>
       <x:c r="AI93" s="46" t="n">
         <x:f>AVERAGE(O93:T93)</x:f>
-        <x:v>4.333333333333333</x:v>
+        <x:v>3.5</x:v>
       </x:c>
       <x:c r="AJ93" s="46" t="n">
         <x:f>AVERAGE(U93:Z93)</x:f>
@@ -11567,21 +11573,21 @@
       </x:c>
       <x:c r="AK93" s="46" t="n">
         <x:f>AVERAGE(AA93:AG93)</x:f>
-        <x:v>4.285714285714286</x:v>
+        <x:v>2.7142857142857144</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="44" t="str">
-        <x:v>Manual-55</x:v>
+        <x:v>Manual-57</x:v>
       </x:c>
       <x:c r="B94" s="44" t="str">
         <x:v>manual</x:v>
       </x:c>
       <x:c r="C94" s="44" t="str">
-        <x:v>45–54</x:v>
+        <x:v>25–34</x:v>
       </x:c>
       <x:c r="D94" s="44" t="str">
-        <x:v>Above 20 years</x:v>
+        <x:v>5–10 years</x:v>
       </x:c>
       <x:c r="E94" s="44" t="str">
         <x:v>Officer</x:v>
@@ -11593,28 +11599,28 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H94" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I94" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="J94" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="K94" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L94" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="M94" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="N94" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="O94" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="P94" s="46" t="n">
         <x:v>5</x:v>
@@ -11623,10 +11629,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="R94" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="S94" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="T94" s="46" t="n">
         <x:v>4</x:v>
@@ -11635,7 +11641,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="V94" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="W94" s="46" t="n">
         <x:v>4</x:v>
@@ -11650,55 +11656,55 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="AA94" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AB94" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AC94" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="AD94" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AE94" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AF94" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AG94" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AH94" s="46" t="n">
         <x:f>AVERAGE(H94:N94)</x:f>
-        <x:v>4.285714285714286</x:v>
+        <x:v>4.571428571428571</x:v>
       </x:c>
       <x:c r="AI94" s="46" t="n">
         <x:f>AVERAGE(O94:T94)</x:f>
-        <x:v>4.333333333333333</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="AJ94" s="46" t="n">
         <x:f>AVERAGE(U94:Z94)</x:f>
-        <x:v>4.333333333333333</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="AK94" s="46" t="n">
         <x:f>AVERAGE(AA94:AG94)</x:f>
-        <x:v>4.714285714285714</x:v>
+        <x:v>4.142857142857143</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="44" t="str">
-        <x:v>Manual-56</x:v>
+        <x:v>Manual-58</x:v>
       </x:c>
       <x:c r="B95" s="44" t="str">
         <x:v>manual</x:v>
       </x:c>
       <x:c r="C95" s="44" t="str">
-        <x:v>25–34</x:v>
+        <x:v>35–44</x:v>
       </x:c>
       <x:c r="D95" s="44" t="str">
-        <x:v>Below 5 years</x:v>
+        <x:v>11–20 years</x:v>
       </x:c>
       <x:c r="E95" s="44" t="str">
         <x:v>Officer</x:v>
@@ -11710,112 +11716,112 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H95" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I95" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J95" s="46" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K95" s="46" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K95" s="46" t="n">
-        <x:v>3</x:v>
-      </x:c>
       <x:c r="L95" s="46" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M95" s="46" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N95" s="46" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O95" s="46" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="M95" s="46" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="N95" s="46" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="O95" s="46" t="n">
-        <x:v>4</x:v>
-      </x:c>
       <x:c r="P95" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Q95" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="R95" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="S95" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="T95" s="46" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U95" s="46" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="U95" s="46" t="n">
-        <x:v>4</x:v>
-      </x:c>
       <x:c r="V95" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="W95" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="X95" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Y95" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="Z95" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AA95" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="AB95" s="46" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AC95" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AD95" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AE95" s="46" t="n">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AF95" s="46" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AG95" s="46" t="n">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AH95" s="46" t="n">
         <x:f>AVERAGE(H95:N95)</x:f>
-        <x:v>2.857142857142857</x:v>
+        <x:v>1.4285714285714286</x:v>
       </x:c>
       <x:c r="AI95" s="46" t="n">
         <x:f>AVERAGE(O95:T95)</x:f>
-        <x:v>3.5</x:v>
+        <x:v>1.6666666666666667</x:v>
       </x:c>
       <x:c r="AJ95" s="46" t="n">
         <x:f>AVERAGE(U95:Z95)</x:f>
-        <x:v>4</x:v>
+        <x:v>4.333333333333333</x:v>
       </x:c>
       <x:c r="AK95" s="46" t="n">
         <x:f>AVERAGE(AA95:AG95)</x:f>
-        <x:v>2.7142857142857144</x:v>
+        <x:v>4.428571428571429</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="44" t="str">
-        <x:v>Manual-57</x:v>
+        <x:v>Manual-60</x:v>
       </x:c>
       <x:c r="B96" s="44" t="str">
         <x:v>manual</x:v>
       </x:c>
       <x:c r="C96" s="44" t="str">
-        <x:v>25–34</x:v>
+        <x:v>35–44</x:v>
       </x:c>
       <x:c r="D96" s="44" t="str">
-        <x:v>5–10 years</x:v>
+        <x:v>11–20 years</x:v>
       </x:c>
       <x:c r="E96" s="44" t="str">
         <x:v>Officer</x:v>
@@ -11830,34 +11836,34 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="I96" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J96" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="K96" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L96" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="M96" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N96" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="O96" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="P96" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Q96" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="R96" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="S96" s="46" t="n">
         <x:v>4</x:v>
@@ -11869,13 +11875,13 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="V96" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="W96" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="X96" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Y96" s="46" t="n">
         <x:v>4</x:v>
@@ -11884,7 +11890,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="AA96" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AB96" s="46" t="n">
         <x:v>4</x:v>
@@ -11893,7 +11899,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="AD96" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AE96" s="46" t="n">
         <x:v>4</x:v>
@@ -11906,15 +11912,15 @@
       </x:c>
       <x:c r="AH96" s="46" t="n">
         <x:f>AVERAGE(H96:N96)</x:f>
-        <x:v>4.571428571428571</x:v>
+        <x:v>3.5714285714285716</x:v>
       </x:c>
       <x:c r="AI96" s="46" t="n">
         <x:f>AVERAGE(O96:T96)</x:f>
-        <x:v>4.5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AJ96" s="46" t="n">
         <x:f>AVERAGE(U96:Z96)</x:f>
-        <x:v>4.5</x:v>
+        <x:v>4.166666666666667</x:v>
       </x:c>
       <x:c r="AK96" s="46" t="n">
         <x:f>AVERAGE(AA96:AG96)</x:f>
@@ -11923,7 +11929,7 @@
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="44" t="str">
-        <x:v>Manual-58</x:v>
+        <x:v>Manual-62</x:v>
       </x:c>
       <x:c r="B97" s="44" t="str">
         <x:v>manual</x:v>
@@ -11944,61 +11950,61 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H97" s="46" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I97" s="46" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J97" s="46" t="n">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="K97" s="46" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L97" s="46" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="M97" s="46" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="N97" s="46" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="O97" s="46" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="P97" s="46" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Q97" s="46" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="R97" s="46" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="S97" s="46" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="T97" s="46" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="U97" s="46" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="V97" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="W97" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="X97" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Y97" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="Z97" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AA97" s="46" t="n">
         <x:v>4</x:v>
@@ -12010,49 +12016,49 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="AD97" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AE97" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AF97" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="AG97" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AH97" s="46" t="n">
         <x:f>AVERAGE(H97:N97)</x:f>
-        <x:v>1.4285714285714286</x:v>
+        <x:v>3.857142857142857</x:v>
       </x:c>
       <x:c r="AI97" s="46" t="n">
         <x:f>AVERAGE(O97:T97)</x:f>
-        <x:v>1.6666666666666667</x:v>
+        <x:v>3.8333333333333335</x:v>
       </x:c>
       <x:c r="AJ97" s="46" t="n">
         <x:f>AVERAGE(U97:Z97)</x:f>
-        <x:v>4.333333333333333</x:v>
+        <x:v>3.8333333333333335</x:v>
       </x:c>
       <x:c r="AK97" s="46" t="n">
         <x:f>AVERAGE(AA97:AG97)</x:f>
-        <x:v>4.428571428571429</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="44" t="str">
-        <x:v>Manual-60</x:v>
+        <x:v>Manual-63</x:v>
       </x:c>
       <x:c r="B98" s="44" t="str">
         <x:v>manual</x:v>
       </x:c>
       <x:c r="C98" s="44" t="str">
-        <x:v>35–44</x:v>
+        <x:v>25–34</x:v>
       </x:c>
       <x:c r="D98" s="44" t="str">
-        <x:v>11–20 years</x:v>
+        <x:v>Below 5 years</x:v>
       </x:c>
       <x:c r="E98" s="44" t="str">
-        <x:v>Officer</x:v>
+        <x:v>Clerical</x:v>
       </x:c>
       <x:c r="F98" s="45" t="n">
         <x:v>0</x:v>
@@ -12064,19 +12070,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="I98" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J98" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="K98" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L98" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M98" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="N98" s="46" t="n">
         <x:v>4</x:v>
@@ -12085,7 +12091,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="P98" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Q98" s="46" t="n">
         <x:v>4</x:v>
@@ -12094,70 +12100,70 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="S98" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T98" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="U98" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="V98" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="W98" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="X98" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Y98" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Z98" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AA98" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="AB98" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AC98" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AD98" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="AE98" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AF98" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AG98" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AH98" s="46" t="n">
         <x:f>AVERAGE(H98:N98)</x:f>
-        <x:v>3.5714285714285716</x:v>
+        <x:v>3.2857142857142856</x:v>
       </x:c>
       <x:c r="AI98" s="46" t="n">
         <x:f>AVERAGE(O98:T98)</x:f>
-        <x:v>4</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="AJ98" s="46" t="n">
         <x:f>AVERAGE(U98:Z98)</x:f>
-        <x:v>4.166666666666667</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AK98" s="46" t="n">
         <x:f>AVERAGE(AA98:AG98)</x:f>
-        <x:v>4.142857142857143</x:v>
+        <x:v>4.857142857142857</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="44" t="str">
-        <x:v>Manual-62</x:v>
+        <x:v>Manual-64</x:v>
       </x:c>
       <x:c r="B99" s="44" t="str">
         <x:v>manual</x:v>
@@ -12166,7 +12172,7 @@
         <x:v>35–44</x:v>
       </x:c>
       <x:c r="D99" s="44" t="str">
-        <x:v>11–20 years</x:v>
+        <x:v>5–10 years</x:v>
       </x:c>
       <x:c r="E99" s="44" t="str">
         <x:v>Officer</x:v>
@@ -12181,16 +12187,16 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="I99" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J99" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="K99" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L99" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="M99" s="46" t="n">
         <x:v>4</x:v>
@@ -12199,28 +12205,28 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="O99" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="P99" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="Q99" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="R99" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="S99" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="T99" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="U99" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="V99" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="W99" s="46" t="n">
         <x:v>4</x:v>
@@ -12229,7 +12235,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="Y99" s="46" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Z99" s="46" t="n">
         <x:v>4</x:v>
@@ -12244,46 +12250,46 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="AD99" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AE99" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AF99" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AG99" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="AH99" s="46" t="n">
         <x:f>AVERAGE(H99:N99)</x:f>
-        <x:v>3.857142857142857</x:v>
+        <x:v>4.285714285714286</x:v>
       </x:c>
       <x:c r="AI99" s="46" t="n">
         <x:f>AVERAGE(O99:T99)</x:f>
-        <x:v>3.8333333333333335</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="AJ99" s="46" t="n">
         <x:f>AVERAGE(U99:Z99)</x:f>
-        <x:v>3.8333333333333335</x:v>
+        <x:v>4.333333333333333</x:v>
       </x:c>
       <x:c r="AK99" s="46" t="n">
         <x:f>AVERAGE(AA99:AG99)</x:f>
-        <x:v>4</x:v>
+        <x:v>4.428571428571429</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="44" t="str">
-        <x:v>Manual-63</x:v>
+        <x:v>Manual-65</x:v>
       </x:c>
       <x:c r="B100" s="44" t="str">
         <x:v>manual</x:v>
       </x:c>
       <x:c r="C100" s="44" t="str">
-        <x:v>25–34</x:v>
+        <x:v>35–44</x:v>
       </x:c>
       <x:c r="D100" s="44" t="str">
-        <x:v>Below 5 years</x:v>
+        <x:v>11–20 years</x:v>
       </x:c>
       <x:c r="E100" s="44" t="str">
         <x:v>Clerical</x:v>
@@ -12295,10 +12301,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H100" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="I100" s="46" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J100" s="46" t="n">
         <x:v>4</x:v>
@@ -12307,25 +12313,25 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="L100" s="46" t="n">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="M100" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="N100" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="O100" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="P100" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Q100" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="R100" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="S100" s="46" t="n">
         <x:v>5</x:v>
@@ -12334,25 +12340,25 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="U100" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="V100" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="W100" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="X100" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="Y100" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Z100" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="AA100" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AB100" s="46" t="n">
         <x:v>5</x:v>
@@ -12364,34 +12370,34 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="AE100" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AF100" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AG100" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="AH100" s="46" t="n">
         <x:f>AVERAGE(H100:N100)</x:f>
-        <x:v>3.2857142857142856</x:v>
+        <x:v>4.571428571428571</x:v>
       </x:c>
       <x:c r="AI100" s="46" t="n">
         <x:f>AVERAGE(O100:T100)</x:f>
-        <x:v>4.5</x:v>
+        <x:v>4.666666666666667</x:v>
       </x:c>
       <x:c r="AJ100" s="46" t="n">
         <x:f>AVERAGE(U100:Z100)</x:f>
-        <x:v>5</x:v>
+        <x:v>4.333333333333333</x:v>
       </x:c>
       <x:c r="AK100" s="46" t="n">
         <x:f>AVERAGE(AA100:AG100)</x:f>
-        <x:v>4.857142857142857</x:v>
+        <x:v>4.714285714285714</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="44" t="str">
-        <x:v>Manual-64</x:v>
+        <x:v>Manual-66</x:v>
       </x:c>
       <x:c r="B101" s="44" t="str">
         <x:v>manual</x:v>
@@ -12400,10 +12406,10 @@
         <x:v>35–44</x:v>
       </x:c>
       <x:c r="D101" s="44" t="str">
-        <x:v>5–10 years</x:v>
+        <x:v>11–20 years</x:v>
       </x:c>
       <x:c r="E101" s="44" t="str">
-        <x:v>Officer</x:v>
+        <x:v>Clerical</x:v>
       </x:c>
       <x:c r="F101" s="45" t="n">
         <x:v>0</x:v>
@@ -12412,7 +12418,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H101" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="I101" s="46" t="n">
         <x:v>5</x:v>
@@ -12421,19 +12427,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="K101" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L101" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="M101" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="N101" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="O101" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="P101" s="46" t="n">
         <x:v>4</x:v>
@@ -12445,25 +12451,25 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="S101" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T101" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="U101" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="V101" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="W101" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="X101" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Y101" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Z101" s="46" t="n">
         <x:v>4</x:v>
@@ -12487,28 +12493,28 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="AG101" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AH101" s="46" t="n">
         <x:f>AVERAGE(H101:N101)</x:f>
-        <x:v>4.285714285714286</x:v>
+        <x:v>4.428571428571429</x:v>
       </x:c>
       <x:c r="AI101" s="46" t="n">
         <x:f>AVERAGE(O101:T101)</x:f>
-        <x:v>4.5</x:v>
+        <x:v>4.333333333333333</x:v>
       </x:c>
       <x:c r="AJ101" s="46" t="n">
         <x:f>AVERAGE(U101:Z101)</x:f>
-        <x:v>4.333333333333333</x:v>
+        <x:v>4.666666666666667</x:v>
       </x:c>
       <x:c r="AK101" s="46" t="n">
         <x:f>AVERAGE(AA101:AG101)</x:f>
-        <x:v>4.428571428571429</x:v>
+        <x:v>4.571428571428571</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="44" t="str">
-        <x:v>Manual-65</x:v>
+        <x:v>Manual-67</x:v>
       </x:c>
       <x:c r="B102" s="44" t="str">
         <x:v>manual</x:v>
@@ -12520,7 +12526,7 @@
         <x:v>11–20 years</x:v>
       </x:c>
       <x:c r="E102" s="44" t="str">
-        <x:v>Clerical</x:v>
+        <x:v>Officer</x:v>
       </x:c>
       <x:c r="F102" s="45" t="n">
         <x:v>0</x:v>
@@ -12535,19 +12541,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="J102" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="K102" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="L102" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="M102" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="N102" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="O102" s="46" t="n">
         <x:v>4</x:v>
@@ -12556,13 +12562,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="Q102" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="R102" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="S102" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="T102" s="46" t="n">
         <x:v>5</x:v>
@@ -12580,13 +12586,13 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="Y102" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Z102" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="AA102" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AB102" s="46" t="n">
         <x:v>5</x:v>
@@ -12595,7 +12601,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="AD102" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AE102" s="46" t="n">
         <x:v>4</x:v>
@@ -12604,28 +12610,28 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="AG102" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AH102" s="46" t="n">
         <x:f>AVERAGE(H102:N102)</x:f>
-        <x:v>4.571428571428571</x:v>
+        <x:v>4.285714285714286</x:v>
       </x:c>
       <x:c r="AI102" s="46" t="n">
         <x:f>AVERAGE(O102:T102)</x:f>
-        <x:v>4.666666666666667</x:v>
+        <x:v>4.166666666666667</x:v>
       </x:c>
       <x:c r="AJ102" s="46" t="n">
         <x:f>AVERAGE(U102:Z102)</x:f>
-        <x:v>4.333333333333333</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="AK102" s="46" t="n">
         <x:f>AVERAGE(AA102:AG102)</x:f>
-        <x:v>4.714285714285714</x:v>
+        <x:v>4.285714285714286</x:v>
       </x:c>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="44" t="str">
-        <x:v>Manual-66</x:v>
+        <x:v>Manual-68</x:v>
       </x:c>
       <x:c r="B103" s="44" t="str">
         <x:v>manual</x:v>
@@ -12652,28 +12658,28 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="J103" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="K103" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L103" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="M103" s="46" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="N103" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="O103" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="P103" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Q103" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="R103" s="46" t="n">
         <x:v>5</x:v>
@@ -12682,7 +12688,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="T103" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="U103" s="46" t="n">
         <x:v>5</x:v>
@@ -12697,19 +12703,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="Y103" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Z103" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AA103" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AB103" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AC103" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AD103" s="46" t="n">
         <x:v>5</x:v>
@@ -12725,33 +12731,33 @@
       </x:c>
       <x:c r="AH103" s="46" t="n">
         <x:f>AVERAGE(H103:N103)</x:f>
-        <x:v>4.428571428571429</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AI103" s="46" t="n">
         <x:f>AVERAGE(O103:T103)</x:f>
-        <x:v>4.333333333333333</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AJ103" s="46" t="n">
         <x:f>AVERAGE(U103:Z103)</x:f>
-        <x:v>4.666666666666667</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AK103" s="46" t="n">
         <x:f>AVERAGE(AA103:AG103)</x:f>
-        <x:v>4.571428571428571</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="44" t="str">
-        <x:v>Manual-67</x:v>
+        <x:v>Manual-70</x:v>
       </x:c>
       <x:c r="B104" s="44" t="str">
         <x:v>manual</x:v>
       </x:c>
       <x:c r="C104" s="44" t="str">
-        <x:v>35–44</x:v>
+        <x:v>25–34</x:v>
       </x:c>
       <x:c r="D104" s="44" t="str">
-        <x:v>11–20 years</x:v>
+        <x:v>Below 5 years</x:v>
       </x:c>
       <x:c r="E104" s="44" t="str">
         <x:v>Officer</x:v>
@@ -12772,13 +12778,13 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="K104" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L104" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="M104" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="N104" s="46" t="n">
         <x:v>4</x:v>
@@ -12796,10 +12802,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="S104" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T104" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="U104" s="46" t="n">
         <x:v>4</x:v>
@@ -12814,7 +12820,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="Y104" s="46" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="Z104" s="46" t="n">
         <x:v>5</x:v>
@@ -12832,17 +12838,17 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="AE104" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AF104" s="46" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="AG104" s="46" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AH104" s="46" t="n">
         <x:f>AVERAGE(H104:N104)</x:f>
-        <x:v>4.285714285714286</x:v>
+        <x:v>4.714285714285714</x:v>
       </x:c>
       <x:c r="AI104" s="46" t="n">
         <x:f>AVERAGE(O104:T104)</x:f>
@@ -12850,251 +12856,95 @@
       </x:c>
       <x:c r="AJ104" s="46" t="n">
         <x:f>AVERAGE(U104:Z104)</x:f>
-        <x:v>4.5</x:v>
+        <x:v>4.166666666666667</x:v>
       </x:c>
       <x:c r="AK104" s="46" t="n">
         <x:f>AVERAGE(AA104:AG104)</x:f>
-        <x:v>4.285714285714286</x:v>
+        <x:v>4.571428571428571</x:v>
       </x:c>
     </x:row>
     <x:row r="105">
-      <x:c r="A105" s="44" t="str">
-        <x:v>Manual-68</x:v>
-      </x:c>
-      <x:c r="B105" s="44" t="str">
-        <x:v>manual</x:v>
-      </x:c>
-      <x:c r="C105" s="44" t="str">
-        <x:v>35–44</x:v>
-      </x:c>
-      <x:c r="D105" s="44" t="str">
-        <x:v>11–20 years</x:v>
-      </x:c>
-      <x:c r="E105" s="44" t="str">
-        <x:v>Clerical</x:v>
-      </x:c>
-      <x:c r="F105" s="45" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G105" s="45" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="I105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="J105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="K105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="L105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="M105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="N105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="O105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="P105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="Q105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="R105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="S105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="T105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="U105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="V105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="W105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="X105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="Y105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="Z105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="AA105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="AB105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="AC105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="AD105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="AE105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="AF105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="AG105" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="AH105" s="46" t="n">
-        <x:f>AVERAGE(H105:N105)</x:f>
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="AI105" s="46" t="n">
-        <x:f>AVERAGE(O105:T105)</x:f>
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="AJ105" s="46" t="n">
-        <x:f>AVERAGE(U105:Z105)</x:f>
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="AK105" s="46" t="n">
-        <x:f>AVERAGE(AA105:AG105)</x:f>
-        <x:v>5</x:v>
-      </x:c>
+      <x:c r="A105" s="44"/>
+      <x:c r="B105" s="44"/>
+      <x:c r="C105" s="44"/>
+      <x:c r="D105" s="44"/>
+      <x:c r="E105" s="44"/>
+      <x:c r="F105" s="45"/>
+      <x:c r="G105" s="45"/>
+      <x:c r="H105" s="46"/>
+      <x:c r="I105" s="46"/>
+      <x:c r="J105" s="46"/>
+      <x:c r="K105" s="46"/>
+      <x:c r="L105" s="46"/>
+      <x:c r="M105" s="46"/>
+      <x:c r="N105" s="46"/>
+      <x:c r="O105" s="46"/>
+      <x:c r="P105" s="46"/>
+      <x:c r="Q105" s="46"/>
+      <x:c r="R105" s="46"/>
+      <x:c r="S105" s="46"/>
+      <x:c r="T105" s="46"/>
+      <x:c r="U105" s="46"/>
+      <x:c r="V105" s="46"/>
+      <x:c r="W105" s="46"/>
+      <x:c r="X105" s="46"/>
+      <x:c r="Y105" s="46"/>
+      <x:c r="Z105" s="46"/>
+      <x:c r="AA105" s="46"/>
+      <x:c r="AB105" s="46"/>
+      <x:c r="AC105" s="46"/>
+      <x:c r="AD105" s="46"/>
+      <x:c r="AE105" s="46"/>
+      <x:c r="AF105" s="46"/>
+      <x:c r="AG105" s="46"/>
+      <x:c r="AH105" s="46"/>
+      <x:c r="AI105" s="46"/>
+      <x:c r="AJ105" s="46"/>
+      <x:c r="AK105" s="46"/>
     </x:row>
     <x:row r="106">
-      <x:c r="A106" s="44" t="str">
-        <x:v>Manual-70</x:v>
-      </x:c>
-      <x:c r="B106" s="44" t="str">
-        <x:v>manual</x:v>
-      </x:c>
-      <x:c r="C106" s="44" t="str">
-        <x:v>25–34</x:v>
-      </x:c>
-      <x:c r="D106" s="44" t="str">
-        <x:v>Below 5 years</x:v>
-      </x:c>
-      <x:c r="E106" s="44" t="str">
-        <x:v>Officer</x:v>
-      </x:c>
-      <x:c r="F106" s="45" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G106" s="45" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H106" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="I106" s="46" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J106" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="K106" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="L106" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="M106" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="N106" s="46" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="O106" s="46" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="P106" s="46" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="Q106" s="46" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="R106" s="46" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="S106" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="T106" s="46" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="U106" s="46" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="V106" s="46" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="W106" s="46" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="X106" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="Y106" s="46" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="Z106" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="AA106" s="46" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="AB106" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="AC106" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="AD106" s="46" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="AE106" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="AF106" s="46" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="AG106" s="46" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="AH106" s="46" t="n">
-        <x:f>AVERAGE(H106:N106)</x:f>
-        <x:v>4.714285714285714</x:v>
-      </x:c>
-      <x:c r="AI106" s="46" t="n">
-        <x:f>AVERAGE(O106:T106)</x:f>
-        <x:v>4.166666666666667</x:v>
-      </x:c>
-      <x:c r="AJ106" s="46" t="n">
-        <x:f>AVERAGE(U106:Z106)</x:f>
-        <x:v>4.166666666666667</x:v>
-      </x:c>
-      <x:c r="AK106" s="46" t="n">
-        <x:f>AVERAGE(AA106:AG106)</x:f>
-        <x:v>4.571428571428571</x:v>
-      </x:c>
+      <x:c r="A106" s="44"/>
+      <x:c r="B106" s="44"/>
+      <x:c r="C106" s="44"/>
+      <x:c r="D106" s="44"/>
+      <x:c r="E106" s="44"/>
+      <x:c r="F106" s="45"/>
+      <x:c r="G106" s="45"/>
+      <x:c r="H106" s="46"/>
+      <x:c r="I106" s="46"/>
+      <x:c r="J106" s="46"/>
+      <x:c r="K106" s="46"/>
+      <x:c r="L106" s="46"/>
+      <x:c r="M106" s="46"/>
+      <x:c r="N106" s="46"/>
+      <x:c r="O106" s="46"/>
+      <x:c r="P106" s="46"/>
+      <x:c r="Q106" s="46"/>
+      <x:c r="R106" s="46"/>
+      <x:c r="S106" s="46"/>
+      <x:c r="T106" s="46"/>
+      <x:c r="U106" s="46"/>
+      <x:c r="V106" s="46"/>
+      <x:c r="W106" s="46"/>
+      <x:c r="X106" s="46"/>
+      <x:c r="Y106" s="46"/>
+      <x:c r="Z106" s="46"/>
+      <x:c r="AA106" s="46"/>
+      <x:c r="AB106" s="46"/>
+      <x:c r="AC106" s="46"/>
+      <x:c r="AD106" s="46"/>
+      <x:c r="AE106" s="46"/>
+      <x:c r="AF106" s="46"/>
+      <x:c r="AG106" s="46"/>
+      <x:c r="AH106" s="46"/>
+      <x:c r="AI106" s="46"/>
+      <x:c r="AJ106" s="46"/>
+      <x:c r="AK106" s="46"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72b14b53943a4953"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ee9a709ba7847c4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17313,7 +17163,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72d1882c5dba47d0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c9bc5765caa4118"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>